<commit_message>
Updated the cross dividing logic on ref-sites and finalized the LDA classifier.
</commit_message>
<xml_diff>
--- a/results/02_taxa_assemblage/MRT_Method/ModelA_CoreOnly/tables/confusion_matrix_unified.xlsx
+++ b/results/02_taxa_assemblage/MRT_Method/ModelA_CoreOnly/tables/confusion_matrix_unified.xlsx
@@ -425,18 +425,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Part 1: Training Resubstitution — Core (n=25)</t>
+          <t>Part 1: Training Resubstitution — Core (n=42)</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
       <c r="C1" t="inlineStr"/>
       <c r="D1" t="inlineStr"/>
+      <c r="E1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr"/>
@@ -455,6 +456,11 @@
           <t>Cluster C2</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Cluster C3</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -466,9 +472,12 @@
         <v>100</v>
       </c>
       <c r="C3" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -479,193 +488,288 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>88</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D4" t="n">
-        <v>7</v>
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
+          <t>Cluster C3</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>96</v>
-      </c>
-      <c r="C5" t="n">
-        <v>18</v>
-      </c>
-      <c r="D5" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
+      <c r="B6" t="n">
+        <v>60</v>
+      </c>
+      <c r="C6" t="n">
+        <v>42</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>Part 2: 5-Fold x 10 Cross-Validation — Core (n=25)</t>
-        </is>
-      </c>
+      <c r="A7" s="1" t="inlineStr"/>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr"/>
-      <c r="B8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Part 2: 5-Fold x 10 Cross-Validation — Core (n=42)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
         <is>
           <t>% Correct</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Cluster C1</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Cluster C2</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>Cluster C1</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>81</v>
-      </c>
-      <c r="C9" t="n">
-        <v>138</v>
-      </c>
-      <c r="D9" t="n">
-        <v>32</v>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Cluster C3</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Cluster C2</t>
+          <t>Cluster C1</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>61</v>
+        <v>86</v>
       </c>
       <c r="C10" t="n">
-        <v>31</v>
+        <v>215</v>
       </c>
       <c r="D10" t="n">
-        <v>49</v>
+        <v>35</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Cluster C2</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>75</v>
+        <v>39</v>
       </c>
       <c r="C11" t="n">
-        <v>169</v>
+        <v>55</v>
       </c>
       <c r="D11" t="n">
-        <v>81</v>
+        <v>35</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Cluster C3</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>77</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Part 3: Held-out Prediction — Peripheral (n=23) + Uncertain (n=2)</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>60</v>
+      </c>
+      <c r="C13" t="n">
+        <v>347</v>
+      </c>
+      <c r="D13" t="n">
+        <v>73</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr"/>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>% Correct</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Cluster C1</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Cluster C2</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
+          <t>Part 3: Held-out Prediction — Peripheral (n=6) + Uncertain (n=2)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>% Correct</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
           <t>Cluster C1</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>86</v>
-      </c>
-      <c r="C15" t="n">
-        <v>12</v>
-      </c>
-      <c r="D15" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Cluster C2</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>100</v>
-      </c>
-      <c r="C16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" t="n">
-        <v>1</v>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Cluster C3</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
+          <t>Cluster C1</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>100</v>
+      </c>
+      <c r="C17" t="n">
+        <v>6</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Cluster C2</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>Cluster C3</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>87</v>
-      </c>
-      <c r="C17" t="n">
-        <v>12</v>
-      </c>
-      <c r="D17" t="n">
-        <v>3</v>
+      <c r="B20" t="n">
+        <v>75</v>
+      </c>
+      <c r="C20" t="n">
+        <v>8</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>